<commit_message>
Correct 82 North Shore Road coordinates
BC0020-26 (80 kW, Devonshire) sat at 32.373,-64.756604 -- about a
kilometre offshore, north of the island, which put an 80 kW marker in
open water. The Department supplied the surveyed position:
32.3056539905629, -64.78817544197068.

Patched as a two-cell edit to the sheet XML rather than by rewriting the
workbook. Loading and saving it with openpyxl re-typed eight numeric
System Capacity cells as text, which silently dropped the published
total from 15,025.02 to 14,866.68 kW: the capacity import counts numeric
cells only, so a change of cell type is a change of published figure.
Every other entry in the archive is copied through byte for byte.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/server/data/Solar Panel Application 2019-now.xlsx
+++ b/server/data/Solar Panel Application 2019-now.xlsx
@@ -61279,10 +61279,10 @@
         <v>28</v>
       </c>
       <c r="P754" s="10">
-        <v>32.372999999999998</v>
+        <v>32.3056539905629</v>
       </c>
       <c r="Q754" s="10">
-        <v>-64.756603999999996</v>
+        <v>-64.78817544197068</v>
       </c>
     </row>
     <row r="755" spans="1:17" ht="90" customHeight="1" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
Stop anchoring blank-district permits to Pembroke
The recovery pass fell back to a parish road-centre anchor when it could not
place a permit, and where the Permit District column was blank or unrecognised
it defaulted that parish to Pembroke. Two rows have no usable district, and one
of them is the Bermuda Airport Solar Farm -- 6,000 kW, about 40% of the
published capacity. It was dragged 11.9 km from St George's into Pembroke and
plotted in the middle of the wrong parish.

A row with no district has no parish to anchor to, so there is nothing to guess
from. Both rows now keep the coordinate they arrived with: the airport returns
to 32.359139, -64.685694 in St George's, and 47 Paynters Hill stays where it
was. The anchor is only used where a real parish is known, which drops it from
41 rows to 39.

Co-Authored-By: Claude Opus 5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/server/data/Solar Panel Application 2019-now.xlsx
+++ b/server/data/Solar Panel Application 2019-now.xlsx
@@ -35753,10 +35753,10 @@
         <v>Yes</v>
       </c>
       <c r="P648">
-        <v>32.3008022</v>
+        <v>32.273322</v>
       </c>
       <c r="Q648">
-        <v>-64.7915912</v>
+        <v>-64.806901</v>
       </c>
     </row>
     <row r="649" xml:space="preserve">
@@ -43339,10 +43339,10 @@
         <v/>
       </c>
       <c r="P786">
-        <v>32.3008022</v>
+        <v>32.359139</v>
       </c>
       <c r="Q786">
-        <v>-64.7915912</v>
+        <v>-64.685694</v>
       </c>
     </row>
     <row r="787" xml:space="preserve">

</xml_diff>